<commit_message>
Regional member sub-pages: Find a Dentist / Pharmacy / Formulary, Disputes, Surprise Billing, Forms Library
- import-member-subpage.js (template member-subpage, 23 URLs): the FAQ topic sections
  with the region's header and footer; the text's closing spacer, the light-blue band,
  hanging bullets and the Forms Library block
- styles/templates/member-subpage.css: the sub-pages' differences from faq.css, and the
  legal-template pages (Disputes and Appeals, the Forms Libraries)
- blocks/forms-library: the source's keyword search and category filter over an
  authored list of forms; a Filter button on phones
- scripts.js: a Template value may list several templates
- import-member-regional.js: each region's Breadcrumb Title for its sub-pages
- Western New York's 69px regional header bar below 992px
- AGENTS.md: notes

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-member-regional.report.xlsx
+++ b/tools/importer/reports/import-member-regional.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="803">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="907">
   <si>
     <t>_reportFile</t>
   </si>
@@ -556,7 +556,7 @@
     <t>member-regional</t>
   </si>
   <si>
-    <t>2026-10-14T13:54:04.032Z</t>
+    <t>2026-10-15T12:50:59.580Z</t>
   </si>
   <si>
     <t>Member Resources | Highmark Blue Cross Blue Shield</t>
@@ -571,7 +571,7 @@
     <t>member/bcbsde</t>
   </si>
   <si>
-    <t>2026-10-14T13:54:20.674Z</t>
+    <t>2026-10-15T12:51:16.650Z</t>
   </si>
   <si>
     <t>Member Resources | Highmark BCBS Delaware</t>
@@ -589,7 +589,7 @@
     <t>member/bcbswny</t>
   </si>
   <si>
-    <t>2026-10-14T13:54:27.187Z</t>
+    <t>2026-10-15T12:51:21.307Z</t>
   </si>
   <si>
     <t>Member Resources | Highmark BCBS Western New York</t>
@@ -604,7 +604,7 @@
     <t>member/bcbswv</t>
   </si>
   <si>
-    <t>2026-10-14T13:54:14.789Z</t>
+    <t>2026-10-15T12:51:11.121Z</t>
   </si>
   <si>
     <t>Member Resources | Highmark BCBS West Virginia</t>
@@ -619,7 +619,7 @@
     <t>member/blueshield</t>
   </si>
   <si>
-    <t>2026-10-14T13:54:09.131Z</t>
+    <t>2026-10-15T12:51:04.987Z</t>
   </si>
   <si>
     <t>Member Resources for Central and Southeastern PA | Highmark Blue Shield</t>
@@ -634,7 +634,7 @@
     <t>member/blueshieldneny</t>
   </si>
   <si>
-    <t>2026-10-14T13:54:33.498Z</t>
+    <t>2026-10-15T12:51:25.952Z</t>
   </si>
   <si>
     <t>Member Resources | Highmark BS Northeastern New York</t>
@@ -1006,6 +1006,321 @@
     <t>https://www.highmark.com/about/our-story/our-businesses?zg=false</t>
   </si>
   <si>
+    <t>member/bcbs/find-a-dentist.report.json</t>
+  </si>
+  <si>
+    <t>["cards-minimal-light-sidenav"]</t>
+  </si>
+  <si>
+    <t>member/bcbs/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member-subpage</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:30:47.485Z</t>
+  </si>
+  <si>
+    <t>Find a Dentist | Highmark Blue Cross Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbs/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member/bcbs/find-a-pharmacy.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbs/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:30:58.736Z</t>
+  </si>
+  <si>
+    <t>Pharmacy Finder | Highmark Blue Cross Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbs/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>member/bcbs/medical-drug-formulary.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbs/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:30:53.290Z</t>
+  </si>
+  <si>
+    <t>Formulary + Prescription Coverage | Highmark BCBS</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbs/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>member/bcbsde/disputes-appeals.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbsde/disputes-appeals</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:47.630Z</t>
+  </si>
+  <si>
+    <t>Dispute and Appeal Process | Highmark BCBS Delaware</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbsde/disputes-appeals</t>
+  </si>
+  <si>
+    <t>member/bcbsde/find-a-dentist.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbsde/find-a-dentist</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:43.145Z</t>
+  </si>
+  <si>
+    <t>Find a Dentist | Highmark BCBS Delaware</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbsde/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member/bcbsde/find-a-pharmacy.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbsde/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:38.258Z</t>
+  </si>
+  <si>
+    <t>Pharmacy Finder | Highmark BCBS Delaware</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbsde/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>member/bcbsde/medical-drug-formulary.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbsde/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:53.932Z</t>
+  </si>
+  <si>
+    <t>Formulary + Prescription Coverage | Highmark BCBS Delaware</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbsde/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>member/bcbswny/find-a-dentist.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswny/find-a-dentist</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:05.520Z</t>
+  </si>
+  <si>
+    <t>Find a Dentist | Highmark BCBS Western NY</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswny/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member/bcbswny/find-a-pharmacy.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswny/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:00.470Z</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswny/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>member/bcbswny/medical-drug-formulary.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswny/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:11.145Z</t>
+  </si>
+  <si>
+    <t>Formulary | Highmark BCBS Western NY</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswny/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>member/bcbswny/surprise-billing.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswny/surprise-billing</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:17.048Z</t>
+  </si>
+  <si>
+    <t>Surprise Billing | Highmark BCBS Western NY</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswny/surprise-billing</t>
+  </si>
+  <si>
+    <t>member/bcbswv/find-a-dentist.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswv/find-a-dentist</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:26.570Z</t>
+  </si>
+  <si>
+    <t>Find a Dentist | Highmark BCBS West Virginia</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswv/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member/bcbswv/find-a-pharmacy.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswv/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:20.719Z</t>
+  </si>
+  <si>
+    <t>Pharmacy Finder | Highmark BCBS West Virginia</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswv/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>member/bcbswv/medical-drug-formulary.report.json</t>
+  </si>
+  <si>
+    <t>member/bcbswv/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:32.639Z</t>
+  </si>
+  <si>
+    <t>Formulary + Prescription Coverage | Highmark BCBS West Virginia</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/bcbswv/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>member/blueshield/find-a-dentist.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshield/find-a-dentist</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:09.798Z</t>
+  </si>
+  <si>
+    <t>Find a Dentist | Highmark Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshield/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member/blueshield/find-a-pharmacy.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshield/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:05.347Z</t>
+  </si>
+  <si>
+    <t>Pharmacy Finder for Central and SE PA| Highmark Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshield/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>member/blueshield/medical-drug-formulary.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshield/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:31:15.215Z</t>
+  </si>
+  <si>
+    <t>Formulary + Prescription Coverage | Highmark Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshield/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/find-a-dentist.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/find-a-dentist</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:29.475Z</t>
+  </si>
+  <si>
+    <t>Find a Dentist | Highmark Blue Shield Northeastern NY</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshieldneny/find-a-dentist</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/find-a-pharmacy.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:23.335Z</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshieldneny/find-a-pharmacy</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/medical-drug-formulary.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:36.063Z</t>
+  </si>
+  <si>
+    <t>Formulary | Highmark Blue Shield Northeastern NY</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshieldneny/medical-drug-formulary</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/surprise-billing.report.json</t>
+  </si>
+  <si>
+    <t>member/blueshieldneny/surprise-billing</t>
+  </si>
+  <si>
+    <t>2026-10-15T12:32:42.598Z</t>
+  </si>
+  <si>
+    <t>Surprise Billing | Highmark Blue Shield Northeastern NY</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/member/blueshieldneny/surprise-billing</t>
+  </si>
+  <si>
     <t>member/member-guide/find-care.report.json</t>
   </si>
   <si>
@@ -1448,9 +1763,6 @@
   </si>
   <si>
     <t>western-pennsylvania/chip/chip-enhanced-member-supports-and-case-management.report.json</t>
-  </si>
-  <si>
-    <t>["cards-minimal-light-sidenav"]</t>
   </si>
   <si>
     <t>western-pennsylvania/chip/chip-enhanced-member-supports-and-case-management</t>
@@ -2808,7 +3120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K141"/>
+  <dimension ref="A1:K162"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -4750,112 +5062,112 @@
         <v>338</v>
       </c>
       <c r="B56" t="s">
+        <v>332</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" t="s">
         <v>339</v>
       </c>
-      <c r="C56" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>334</v>
+      </c>
+      <c r="I56" t="s">
         <v>340</v>
       </c>
-      <c r="G56" t="s">
-        <v>15</v>
-      </c>
-      <c r="H56" t="s">
+      <c r="J56" t="s">
         <v>341</v>
       </c>
-      <c r="I56" t="s">
+      <c r="K56" t="s">
         <v>342</v>
-      </c>
-      <c r="J56" t="s">
-        <v>343</v>
-      </c>
-      <c r="K56" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>343</v>
+      </c>
+      <c r="B57" t="s">
+        <v>332</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F57" t="s">
+        <v>344</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" t="s">
+        <v>334</v>
+      </c>
+      <c r="I57" t="s">
         <v>345</v>
       </c>
-      <c r="B57" t="s">
+      <c r="J57" t="s">
         <v>346</v>
       </c>
-      <c r="C57" t="s">
-        <v>13</v>
-      </c>
-      <c r="D57" t="s">
-        <v>13</v>
-      </c>
-      <c r="E57" t="s">
-        <v>13</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="K57" t="s">
         <v>347</v>
-      </c>
-      <c r="G57" t="s">
-        <v>15</v>
-      </c>
-      <c r="H57" t="s">
-        <v>348</v>
-      </c>
-      <c r="I57" t="s">
-        <v>349</v>
-      </c>
-      <c r="J57" t="s">
-        <v>350</v>
-      </c>
-      <c r="K57" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>348</v>
+      </c>
+      <c r="B58" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" t="s">
+        <v>13</v>
+      </c>
+      <c r="E58" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" t="s">
+        <v>349</v>
+      </c>
+      <c r="G58" t="s">
+        <v>15</v>
+      </c>
+      <c r="H58" t="s">
+        <v>334</v>
+      </c>
+      <c r="I58" t="s">
+        <v>350</v>
+      </c>
+      <c r="J58" t="s">
+        <v>351</v>
+      </c>
+      <c r="K58" t="s">
         <v>352</v>
-      </c>
-      <c r="B58" t="s">
-        <v>353</v>
-      </c>
-      <c r="C58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D58" t="s">
-        <v>13</v>
-      </c>
-      <c r="E58" t="s">
-        <v>13</v>
-      </c>
-      <c r="F58" t="s">
-        <v>354</v>
-      </c>
-      <c r="G58" t="s">
-        <v>15</v>
-      </c>
-      <c r="H58" t="s">
-        <v>341</v>
-      </c>
-      <c r="I58" t="s">
-        <v>355</v>
-      </c>
-      <c r="J58" t="s">
-        <v>356</v>
-      </c>
-      <c r="K58" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="B59" t="s">
-        <v>359</v>
+        <v>332</v>
       </c>
       <c r="C59" t="s">
         <v>13</v>
@@ -4867,30 +5179,30 @@
         <v>13</v>
       </c>
       <c r="F59" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="G59" t="s">
         <v>15</v>
       </c>
       <c r="H59" t="s">
-        <v>361</v>
+        <v>334</v>
       </c>
       <c r="I59" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="J59" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="K59" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="B60" t="s">
-        <v>109</v>
+        <v>332</v>
       </c>
       <c r="C60" t="s">
         <v>13</v>
@@ -4902,30 +5214,30 @@
         <v>13</v>
       </c>
       <c r="F60" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="G60" t="s">
         <v>15</v>
       </c>
       <c r="H60" t="s">
-        <v>367</v>
+        <v>334</v>
       </c>
       <c r="I60" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="J60" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="K60" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="B61" t="s">
-        <v>109</v>
+        <v>332</v>
       </c>
       <c r="C61" t="s">
         <v>13</v>
@@ -4937,30 +5249,30 @@
         <v>13</v>
       </c>
       <c r="F61" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="G61" t="s">
         <v>15</v>
       </c>
       <c r="H61" t="s">
+        <v>334</v>
+      </c>
+      <c r="I61" t="s">
+        <v>365</v>
+      </c>
+      <c r="J61" t="s">
+        <v>366</v>
+      </c>
+      <c r="K61" t="s">
         <v>367</v>
-      </c>
-      <c r="I61" t="s">
-        <v>373</v>
-      </c>
-      <c r="J61" t="s">
-        <v>374</v>
-      </c>
-      <c r="K61" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="B62" t="s">
-        <v>377</v>
+        <v>332</v>
       </c>
       <c r="C62" t="s">
         <v>13</v>
@@ -4972,30 +5284,30 @@
         <v>13</v>
       </c>
       <c r="F62" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="G62" t="s">
         <v>15</v>
       </c>
       <c r="H62" t="s">
-        <v>379</v>
+        <v>334</v>
       </c>
       <c r="I62" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="J62" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="K62" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="B63" t="s">
-        <v>384</v>
+        <v>332</v>
       </c>
       <c r="C63" t="s">
         <v>13</v>
@@ -5007,30 +5319,30 @@
         <v>13</v>
       </c>
       <c r="F63" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="G63" t="s">
         <v>15</v>
       </c>
       <c r="H63" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="I63" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="J63" t="s">
-        <v>387</v>
+        <v>341</v>
       </c>
       <c r="K63" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="B64" t="s">
-        <v>390</v>
+        <v>332</v>
       </c>
       <c r="C64" t="s">
         <v>13</v>
@@ -5042,30 +5354,30 @@
         <v>13</v>
       </c>
       <c r="F64" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="G64" t="s">
         <v>15</v>
       </c>
       <c r="H64" t="s">
-        <v>274</v>
+        <v>334</v>
       </c>
       <c r="I64" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="J64" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
       <c r="K64" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>395</v>
+        <v>382</v>
       </c>
       <c r="B65" t="s">
-        <v>390</v>
+        <v>332</v>
       </c>
       <c r="C65" t="s">
         <v>13</v>
@@ -5077,65 +5389,65 @@
         <v>13</v>
       </c>
       <c r="F65" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="G65" t="s">
         <v>15</v>
       </c>
       <c r="H65" t="s">
-        <v>274</v>
+        <v>334</v>
       </c>
       <c r="I65" t="s">
-        <v>397</v>
+        <v>384</v>
       </c>
       <c r="J65" t="s">
-        <v>398</v>
+        <v>385</v>
       </c>
       <c r="K65" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>400</v>
+        <v>387</v>
       </c>
       <c r="B66" t="s">
+        <v>332</v>
+      </c>
+      <c r="C66" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" t="s">
+        <v>13</v>
+      </c>
+      <c r="E66" t="s">
+        <v>13</v>
+      </c>
+      <c r="F66" t="s">
+        <v>388</v>
+      </c>
+      <c r="G66" t="s">
+        <v>15</v>
+      </c>
+      <c r="H66" t="s">
+        <v>334</v>
+      </c>
+      <c r="I66" t="s">
+        <v>389</v>
+      </c>
+      <c r="J66" t="s">
         <v>390</v>
       </c>
-      <c r="C66" t="s">
-        <v>13</v>
-      </c>
-      <c r="D66" t="s">
-        <v>13</v>
-      </c>
-      <c r="E66" t="s">
-        <v>13</v>
-      </c>
-      <c r="F66" t="s">
-        <v>401</v>
-      </c>
-      <c r="G66" t="s">
-        <v>15</v>
-      </c>
-      <c r="H66" t="s">
-        <v>274</v>
-      </c>
-      <c r="I66" t="s">
-        <v>402</v>
-      </c>
-      <c r="J66" t="s">
-        <v>403</v>
-      </c>
       <c r="K66" t="s">
-        <v>404</v>
+        <v>391</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>405</v>
+        <v>392</v>
       </c>
       <c r="B67" t="s">
-        <v>406</v>
+        <v>332</v>
       </c>
       <c r="C67" t="s">
         <v>13</v>
@@ -5147,30 +5459,30 @@
         <v>13</v>
       </c>
       <c r="F67" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="G67" t="s">
         <v>15</v>
       </c>
       <c r="H67" t="s">
-        <v>274</v>
+        <v>334</v>
       </c>
       <c r="I67" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
       <c r="J67" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="K67" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="B68" t="s">
-        <v>412</v>
+        <v>332</v>
       </c>
       <c r="C68" t="s">
         <v>13</v>
@@ -5182,30 +5494,30 @@
         <v>13</v>
       </c>
       <c r="F68" t="s">
-        <v>413</v>
+        <v>398</v>
       </c>
       <c r="G68" t="s">
         <v>15</v>
       </c>
       <c r="H68" t="s">
-        <v>274</v>
+        <v>334</v>
       </c>
       <c r="I68" t="s">
-        <v>414</v>
+        <v>399</v>
       </c>
       <c r="J68" t="s">
-        <v>415</v>
+        <v>400</v>
       </c>
       <c r="K68" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="B69" t="s">
-        <v>390</v>
+        <v>332</v>
       </c>
       <c r="C69" t="s">
         <v>13</v>
@@ -5217,30 +5529,30 @@
         <v>13</v>
       </c>
       <c r="F69" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G69" t="s">
         <v>15</v>
       </c>
       <c r="H69" t="s">
-        <v>274</v>
+        <v>334</v>
       </c>
       <c r="I69" t="s">
-        <v>419</v>
+        <v>404</v>
       </c>
       <c r="J69" t="s">
-        <v>420</v>
+        <v>405</v>
       </c>
       <c r="K69" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="B70" t="s">
-        <v>109</v>
+        <v>332</v>
       </c>
       <c r="C70" t="s">
         <v>13</v>
@@ -5252,30 +5564,30 @@
         <v>13</v>
       </c>
       <c r="F70" t="s">
-        <v>423</v>
+        <v>408</v>
       </c>
       <c r="G70" t="s">
         <v>15</v>
       </c>
       <c r="H70" t="s">
-        <v>424</v>
+        <v>334</v>
       </c>
       <c r="I70" t="s">
-        <v>425</v>
+        <v>409</v>
       </c>
       <c r="J70" t="s">
-        <v>426</v>
+        <v>410</v>
       </c>
       <c r="K70" t="s">
-        <v>427</v>
+        <v>411</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>428</v>
+        <v>412</v>
       </c>
       <c r="B71" t="s">
-        <v>429</v>
+        <v>332</v>
       </c>
       <c r="C71" t="s">
         <v>13</v>
@@ -5287,30 +5599,30 @@
         <v>13</v>
       </c>
       <c r="F71" t="s">
-        <v>430</v>
+        <v>413</v>
       </c>
       <c r="G71" t="s">
         <v>15</v>
       </c>
       <c r="H71" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="I71" t="s">
-        <v>431</v>
+        <v>414</v>
       </c>
       <c r="J71" t="s">
-        <v>432</v>
+        <v>415</v>
       </c>
       <c r="K71" t="s">
-        <v>433</v>
+        <v>416</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>434</v>
+        <v>417</v>
       </c>
       <c r="B72" t="s">
-        <v>435</v>
+        <v>332</v>
       </c>
       <c r="C72" t="s">
         <v>13</v>
@@ -5322,30 +5634,30 @@
         <v>13</v>
       </c>
       <c r="F72" t="s">
-        <v>436</v>
+        <v>418</v>
       </c>
       <c r="G72" t="s">
         <v>15</v>
       </c>
       <c r="H72" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="I72" t="s">
-        <v>437</v>
+        <v>419</v>
       </c>
       <c r="J72" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="K72" t="s">
-        <v>439</v>
+        <v>421</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>440</v>
+        <v>422</v>
       </c>
       <c r="B73" t="s">
-        <v>429</v>
+        <v>332</v>
       </c>
       <c r="C73" t="s">
         <v>13</v>
@@ -5357,30 +5669,30 @@
         <v>13</v>
       </c>
       <c r="F73" t="s">
-        <v>441</v>
+        <v>423</v>
       </c>
       <c r="G73" t="s">
         <v>15</v>
       </c>
       <c r="H73" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="I73" t="s">
-        <v>442</v>
+        <v>424</v>
       </c>
       <c r="J73" t="s">
-        <v>443</v>
+        <v>341</v>
       </c>
       <c r="K73" t="s">
-        <v>444</v>
+        <v>425</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>445</v>
+        <v>426</v>
       </c>
       <c r="B74" t="s">
-        <v>435</v>
+        <v>332</v>
       </c>
       <c r="C74" t="s">
         <v>13</v>
@@ -5392,33 +5704,33 @@
         <v>13</v>
       </c>
       <c r="F74" t="s">
-        <v>446</v>
+        <v>427</v>
       </c>
       <c r="G74" t="s">
         <v>15</v>
       </c>
       <c r="H74" t="s">
-        <v>261</v>
+        <v>334</v>
       </c>
       <c r="I74" t="s">
-        <v>447</v>
+        <v>428</v>
       </c>
       <c r="J74" t="s">
-        <v>448</v>
+        <v>429</v>
       </c>
       <c r="K74" t="s">
-        <v>449</v>
+        <v>430</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>450</v>
+        <v>431</v>
       </c>
       <c r="B75" t="s">
-        <v>21</v>
+        <v>332</v>
       </c>
       <c r="C75" t="s">
-        <v>451</v>
+        <v>13</v>
       </c>
       <c r="D75" t="s">
         <v>13</v>
@@ -5427,33 +5739,33 @@
         <v>13</v>
       </c>
       <c r="F75" t="s">
-        <v>452</v>
+        <v>432</v>
       </c>
       <c r="G75" t="s">
         <v>15</v>
       </c>
       <c r="H75" t="s">
-        <v>453</v>
+        <v>334</v>
       </c>
       <c r="I75" t="s">
-        <v>454</v>
+        <v>433</v>
       </c>
       <c r="J75" t="s">
-        <v>455</v>
+        <v>434</v>
       </c>
       <c r="K75" t="s">
-        <v>456</v>
+        <v>435</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>457</v>
+        <v>436</v>
       </c>
       <c r="B76" t="s">
-        <v>21</v>
+        <v>437</v>
       </c>
       <c r="C76" t="s">
-        <v>458</v>
+        <v>13</v>
       </c>
       <c r="D76" t="s">
         <v>13</v>
@@ -5462,65 +5774,65 @@
         <v>13</v>
       </c>
       <c r="F76" t="s">
-        <v>459</v>
+        <v>438</v>
       </c>
       <c r="G76" t="s">
         <v>15</v>
       </c>
       <c r="H76" t="s">
-        <v>453</v>
+        <v>439</v>
       </c>
       <c r="I76" t="s">
-        <v>460</v>
+        <v>440</v>
       </c>
       <c r="J76" t="s">
-        <v>461</v>
+        <v>441</v>
       </c>
       <c r="K76" t="s">
-        <v>462</v>
+        <v>442</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>463</v>
+        <v>443</v>
       </c>
       <c r="B77" t="s">
-        <v>21</v>
+        <v>444</v>
       </c>
       <c r="C77" t="s">
-        <v>464</v>
+        <v>13</v>
       </c>
       <c r="D77" t="s">
         <v>13</v>
       </c>
       <c r="E77" t="s">
-        <v>465</v>
+        <v>13</v>
       </c>
       <c r="F77" t="s">
-        <v>466</v>
+        <v>445</v>
       </c>
       <c r="G77" t="s">
         <v>15</v>
       </c>
       <c r="H77" t="s">
-        <v>467</v>
+        <v>446</v>
       </c>
       <c r="I77" t="s">
-        <v>468</v>
+        <v>447</v>
       </c>
       <c r="J77" t="s">
-        <v>469</v>
+        <v>448</v>
       </c>
       <c r="K77" t="s">
-        <v>470</v>
+        <v>449</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>471</v>
+        <v>450</v>
       </c>
       <c r="B78" t="s">
-        <v>472</v>
+        <v>451</v>
       </c>
       <c r="C78" t="s">
         <v>13</v>
@@ -5532,30 +5844,30 @@
         <v>13</v>
       </c>
       <c r="F78" t="s">
-        <v>473</v>
+        <v>452</v>
       </c>
       <c r="G78" t="s">
         <v>15</v>
       </c>
       <c r="H78" t="s">
-        <v>474</v>
+        <v>453</v>
       </c>
       <c r="I78" t="s">
-        <v>475</v>
+        <v>454</v>
       </c>
       <c r="J78" t="s">
-        <v>476</v>
+        <v>455</v>
       </c>
       <c r="K78" t="s">
-        <v>477</v>
+        <v>456</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>478</v>
+        <v>457</v>
       </c>
       <c r="B79" t="s">
-        <v>479</v>
+        <v>458</v>
       </c>
       <c r="C79" t="s">
         <v>13</v>
@@ -5567,30 +5879,30 @@
         <v>13</v>
       </c>
       <c r="F79" t="s">
-        <v>480</v>
+        <v>459</v>
       </c>
       <c r="G79" t="s">
         <v>15</v>
       </c>
       <c r="H79" t="s">
-        <v>474</v>
+        <v>446</v>
       </c>
       <c r="I79" t="s">
-        <v>481</v>
+        <v>460</v>
       </c>
       <c r="J79" t="s">
-        <v>482</v>
+        <v>461</v>
       </c>
       <c r="K79" t="s">
-        <v>483</v>
+        <v>462</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>484</v>
+        <v>463</v>
       </c>
       <c r="B80" t="s">
-        <v>479</v>
+        <v>464</v>
       </c>
       <c r="C80" t="s">
         <v>13</v>
@@ -5602,30 +5914,30 @@
         <v>13</v>
       </c>
       <c r="F80" t="s">
-        <v>485</v>
+        <v>465</v>
       </c>
       <c r="G80" t="s">
         <v>15</v>
       </c>
       <c r="H80" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="I80" t="s">
-        <v>486</v>
+        <v>467</v>
       </c>
       <c r="J80" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="K80" t="s">
-        <v>488</v>
+        <v>469</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>489</v>
+        <v>470</v>
       </c>
       <c r="B81" t="s">
-        <v>479</v>
+        <v>109</v>
       </c>
       <c r="C81" t="s">
         <v>13</v>
@@ -5637,30 +5949,30 @@
         <v>13</v>
       </c>
       <c r="F81" t="s">
-        <v>490</v>
+        <v>471</v>
       </c>
       <c r="G81" t="s">
         <v>15</v>
       </c>
       <c r="H81" t="s">
+        <v>472</v>
+      </c>
+      <c r="I81" t="s">
+        <v>473</v>
+      </c>
+      <c r="J81" t="s">
         <v>474</v>
       </c>
-      <c r="I81" t="s">
-        <v>491</v>
-      </c>
-      <c r="J81" t="s">
-        <v>492</v>
-      </c>
       <c r="K81" t="s">
-        <v>493</v>
+        <v>475</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>494</v>
+        <v>476</v>
       </c>
       <c r="B82" t="s">
-        <v>495</v>
+        <v>109</v>
       </c>
       <c r="C82" t="s">
         <v>13</v>
@@ -5672,30 +5984,30 @@
         <v>13</v>
       </c>
       <c r="F82" t="s">
-        <v>496</v>
+        <v>477</v>
       </c>
       <c r="G82" t="s">
         <v>15</v>
       </c>
       <c r="H82" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="I82" t="s">
-        <v>497</v>
+        <v>478</v>
       </c>
       <c r="J82" t="s">
-        <v>498</v>
+        <v>479</v>
       </c>
       <c r="K82" t="s">
-        <v>499</v>
+        <v>480</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>500</v>
+        <v>481</v>
       </c>
       <c r="B83" t="s">
-        <v>501</v>
+        <v>482</v>
       </c>
       <c r="C83" t="s">
         <v>13</v>
@@ -5707,30 +6019,30 @@
         <v>13</v>
       </c>
       <c r="F83" t="s">
-        <v>502</v>
+        <v>483</v>
       </c>
       <c r="G83" t="s">
         <v>15</v>
       </c>
       <c r="H83" t="s">
-        <v>503</v>
+        <v>484</v>
       </c>
       <c r="I83" t="s">
-        <v>504</v>
+        <v>485</v>
       </c>
       <c r="J83" t="s">
-        <v>505</v>
+        <v>486</v>
       </c>
       <c r="K83" t="s">
-        <v>506</v>
+        <v>487</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>507</v>
+        <v>488</v>
       </c>
       <c r="B84" t="s">
-        <v>501</v>
+        <v>489</v>
       </c>
       <c r="C84" t="s">
         <v>13</v>
@@ -5742,30 +6054,30 @@
         <v>13</v>
       </c>
       <c r="F84" t="s">
-        <v>508</v>
+        <v>490</v>
       </c>
       <c r="G84" t="s">
         <v>15</v>
       </c>
       <c r="H84" t="s">
-        <v>503</v>
+        <v>261</v>
       </c>
       <c r="I84" t="s">
-        <v>509</v>
+        <v>491</v>
       </c>
       <c r="J84" t="s">
-        <v>510</v>
+        <v>492</v>
       </c>
       <c r="K84" t="s">
-        <v>511</v>
+        <v>493</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>512</v>
+        <v>494</v>
       </c>
       <c r="B85" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="C85" t="s">
         <v>13</v>
@@ -5777,65 +6089,65 @@
         <v>13</v>
       </c>
       <c r="F85" t="s">
-        <v>513</v>
+        <v>496</v>
       </c>
       <c r="G85" t="s">
         <v>15</v>
       </c>
       <c r="H85" t="s">
-        <v>503</v>
+        <v>274</v>
       </c>
       <c r="I85" t="s">
-        <v>514</v>
+        <v>497</v>
       </c>
       <c r="J85" t="s">
-        <v>515</v>
+        <v>498</v>
       </c>
       <c r="K85" t="s">
-        <v>516</v>
+        <v>499</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>517</v>
+        <v>500</v>
       </c>
       <c r="B86" t="s">
+        <v>495</v>
+      </c>
+      <c r="C86" t="s">
+        <v>13</v>
+      </c>
+      <c r="D86" t="s">
+        <v>13</v>
+      </c>
+      <c r="E86" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" t="s">
         <v>501</v>
       </c>
-      <c r="C86" t="s">
-        <v>13</v>
-      </c>
-      <c r="D86" t="s">
-        <v>13</v>
-      </c>
-      <c r="E86" t="s">
-        <v>13</v>
-      </c>
-      <c r="F86" t="s">
-        <v>518</v>
-      </c>
       <c r="G86" t="s">
         <v>15</v>
       </c>
       <c r="H86" t="s">
+        <v>274</v>
+      </c>
+      <c r="I86" t="s">
+        <v>502</v>
+      </c>
+      <c r="J86" t="s">
         <v>503</v>
       </c>
-      <c r="I86" t="s">
-        <v>519</v>
-      </c>
-      <c r="J86" t="s">
-        <v>520</v>
-      </c>
       <c r="K86" t="s">
-        <v>214</v>
+        <v>504</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>521</v>
+        <v>505</v>
       </c>
       <c r="B87" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="C87" t="s">
         <v>13</v>
@@ -5847,30 +6159,30 @@
         <v>13</v>
       </c>
       <c r="F87" t="s">
-        <v>522</v>
+        <v>506</v>
       </c>
       <c r="G87" t="s">
         <v>15</v>
       </c>
       <c r="H87" t="s">
-        <v>503</v>
+        <v>274</v>
       </c>
       <c r="I87" t="s">
-        <v>523</v>
+        <v>507</v>
       </c>
       <c r="J87" t="s">
-        <v>13</v>
+        <v>508</v>
       </c>
       <c r="K87" t="s">
-        <v>524</v>
+        <v>509</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>525</v>
+        <v>510</v>
       </c>
       <c r="B88" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="C88" t="s">
         <v>13</v>
@@ -5882,30 +6194,30 @@
         <v>13</v>
       </c>
       <c r="F88" t="s">
-        <v>526</v>
+        <v>512</v>
       </c>
       <c r="G88" t="s">
         <v>15</v>
       </c>
       <c r="H88" t="s">
-        <v>503</v>
+        <v>274</v>
       </c>
       <c r="I88" t="s">
-        <v>527</v>
+        <v>513</v>
       </c>
       <c r="J88" t="s">
-        <v>13</v>
+        <v>514</v>
       </c>
       <c r="K88" t="s">
-        <v>528</v>
+        <v>515</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>529</v>
+        <v>516</v>
       </c>
       <c r="B89" t="s">
-        <v>501</v>
+        <v>517</v>
       </c>
       <c r="C89" t="s">
         <v>13</v>
@@ -5917,30 +6229,30 @@
         <v>13</v>
       </c>
       <c r="F89" t="s">
-        <v>530</v>
+        <v>518</v>
       </c>
       <c r="G89" t="s">
         <v>15</v>
       </c>
       <c r="H89" t="s">
-        <v>503</v>
+        <v>274</v>
       </c>
       <c r="I89" t="s">
-        <v>531</v>
+        <v>519</v>
       </c>
       <c r="J89" t="s">
-        <v>13</v>
+        <v>520</v>
       </c>
       <c r="K89" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="B90" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="C90" t="s">
         <v>13</v>
@@ -5952,30 +6264,30 @@
         <v>13</v>
       </c>
       <c r="F90" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
       <c r="G90" t="s">
         <v>15</v>
       </c>
       <c r="H90" t="s">
-        <v>503</v>
+        <v>274</v>
       </c>
       <c r="I90" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
       <c r="J90" t="s">
-        <v>536</v>
+        <v>525</v>
       </c>
       <c r="K90" t="s">
-        <v>537</v>
+        <v>526</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>538</v>
+        <v>527</v>
       </c>
       <c r="B91" t="s">
-        <v>501</v>
+        <v>109</v>
       </c>
       <c r="C91" t="s">
         <v>13</v>
@@ -5987,30 +6299,30 @@
         <v>13</v>
       </c>
       <c r="F91" t="s">
-        <v>539</v>
+        <v>528</v>
       </c>
       <c r="G91" t="s">
         <v>15</v>
       </c>
       <c r="H91" t="s">
-        <v>503</v>
+        <v>529</v>
       </c>
       <c r="I91" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="J91" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="K91" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>543</v>
+        <v>533</v>
       </c>
       <c r="B92" t="s">
-        <v>501</v>
+        <v>534</v>
       </c>
       <c r="C92" t="s">
         <v>13</v>
@@ -6022,30 +6334,30 @@
         <v>13</v>
       </c>
       <c r="F92" t="s">
-        <v>544</v>
+        <v>535</v>
       </c>
       <c r="G92" t="s">
         <v>15</v>
       </c>
       <c r="H92" t="s">
-        <v>503</v>
+        <v>261</v>
       </c>
       <c r="I92" t="s">
-        <v>545</v>
+        <v>536</v>
       </c>
       <c r="J92" t="s">
-        <v>13</v>
+        <v>537</v>
       </c>
       <c r="K92" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="B93" t="s">
-        <v>501</v>
+        <v>540</v>
       </c>
       <c r="C93" t="s">
         <v>13</v>
@@ -6057,30 +6369,30 @@
         <v>13</v>
       </c>
       <c r="F93" t="s">
-        <v>548</v>
+        <v>541</v>
       </c>
       <c r="G93" t="s">
         <v>15</v>
       </c>
       <c r="H93" t="s">
-        <v>503</v>
+        <v>261</v>
       </c>
       <c r="I93" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
       <c r="J93" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="K93" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="B94" t="s">
-        <v>501</v>
+        <v>534</v>
       </c>
       <c r="C94" t="s">
         <v>13</v>
@@ -6092,30 +6404,30 @@
         <v>13</v>
       </c>
       <c r="F94" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="G94" t="s">
         <v>15</v>
       </c>
       <c r="H94" t="s">
-        <v>503</v>
+        <v>261</v>
       </c>
       <c r="I94" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="J94" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="K94" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="B95" t="s">
-        <v>501</v>
+        <v>540</v>
       </c>
       <c r="C95" t="s">
         <v>13</v>
@@ -6127,135 +6439,135 @@
         <v>13</v>
       </c>
       <c r="F95" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="G95" t="s">
         <v>15</v>
       </c>
       <c r="H95" t="s">
-        <v>503</v>
+        <v>261</v>
       </c>
       <c r="I95" t="s">
-        <v>559</v>
+        <v>552</v>
       </c>
       <c r="J95" t="s">
-        <v>13</v>
+        <v>553</v>
       </c>
       <c r="K95" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>555</v>
+      </c>
+      <c r="B96" t="s">
+        <v>21</v>
+      </c>
+      <c r="C96" t="s">
+        <v>556</v>
+      </c>
+      <c r="D96" t="s">
+        <v>13</v>
+      </c>
+      <c r="E96" t="s">
+        <v>13</v>
+      </c>
+      <c r="F96" t="s">
+        <v>557</v>
+      </c>
+      <c r="G96" t="s">
+        <v>15</v>
+      </c>
+      <c r="H96" t="s">
+        <v>558</v>
+      </c>
+      <c r="I96" t="s">
+        <v>559</v>
+      </c>
+      <c r="J96" t="s">
+        <v>560</v>
+      </c>
+      <c r="K96" t="s">
         <v>561</v>
-      </c>
-      <c r="B96" t="s">
-        <v>501</v>
-      </c>
-      <c r="C96" t="s">
-        <v>13</v>
-      </c>
-      <c r="D96" t="s">
-        <v>13</v>
-      </c>
-      <c r="E96" t="s">
-        <v>13</v>
-      </c>
-      <c r="F96" t="s">
-        <v>562</v>
-      </c>
-      <c r="G96" t="s">
-        <v>15</v>
-      </c>
-      <c r="H96" t="s">
-        <v>503</v>
-      </c>
-      <c r="I96" t="s">
-        <v>563</v>
-      </c>
-      <c r="J96" t="s">
-        <v>564</v>
-      </c>
-      <c r="K96" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>562</v>
+      </c>
+      <c r="B97" t="s">
+        <v>21</v>
+      </c>
+      <c r="C97" t="s">
+        <v>563</v>
+      </c>
+      <c r="D97" t="s">
+        <v>13</v>
+      </c>
+      <c r="E97" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" t="s">
+        <v>564</v>
+      </c>
+      <c r="G97" t="s">
+        <v>15</v>
+      </c>
+      <c r="H97" t="s">
+        <v>558</v>
+      </c>
+      <c r="I97" t="s">
+        <v>565</v>
+      </c>
+      <c r="J97" t="s">
         <v>566</v>
       </c>
-      <c r="B97" t="s">
-        <v>501</v>
-      </c>
-      <c r="C97" t="s">
-        <v>13</v>
-      </c>
-      <c r="D97" t="s">
-        <v>13</v>
-      </c>
-      <c r="E97" t="s">
-        <v>13</v>
-      </c>
-      <c r="F97" t="s">
+      <c r="K97" t="s">
         <v>567</v>
-      </c>
-      <c r="G97" t="s">
-        <v>15</v>
-      </c>
-      <c r="H97" t="s">
-        <v>503</v>
-      </c>
-      <c r="I97" t="s">
-        <v>568</v>
-      </c>
-      <c r="J97" t="s">
-        <v>569</v>
-      </c>
-      <c r="K97" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>568</v>
+      </c>
+      <c r="B98" t="s">
+        <v>21</v>
+      </c>
+      <c r="C98" t="s">
+        <v>569</v>
+      </c>
+      <c r="D98" t="s">
+        <v>13</v>
+      </c>
+      <c r="E98" t="s">
+        <v>570</v>
+      </c>
+      <c r="F98" t="s">
         <v>571</v>
       </c>
-      <c r="B98" t="s">
-        <v>501</v>
-      </c>
-      <c r="C98" t="s">
-        <v>13</v>
-      </c>
-      <c r="D98" t="s">
-        <v>13</v>
-      </c>
-      <c r="E98" t="s">
-        <v>13</v>
-      </c>
-      <c r="F98" t="s">
+      <c r="G98" t="s">
+        <v>15</v>
+      </c>
+      <c r="H98" t="s">
         <v>572</v>
-      </c>
-      <c r="G98" t="s">
-        <v>15</v>
-      </c>
-      <c r="H98" t="s">
-        <v>503</v>
       </c>
       <c r="I98" t="s">
         <v>573</v>
       </c>
       <c r="J98" t="s">
-        <v>13</v>
+        <v>574</v>
       </c>
       <c r="K98" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B99" t="s">
-        <v>13</v>
+        <v>577</v>
       </c>
       <c r="C99" t="s">
         <v>13</v>
@@ -6267,30 +6579,30 @@
         <v>13</v>
       </c>
       <c r="F99" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="G99" t="s">
         <v>15</v>
       </c>
       <c r="H99" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I99" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="J99" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="K99" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B100" t="s">
-        <v>13</v>
+        <v>332</v>
       </c>
       <c r="C100" t="s">
         <v>13</v>
@@ -6302,30 +6614,30 @@
         <v>13</v>
       </c>
       <c r="F100" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="G100" t="s">
         <v>15</v>
       </c>
       <c r="H100" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I100" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="J100" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="K100" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B101" t="s">
-        <v>13</v>
+        <v>332</v>
       </c>
       <c r="C101" t="s">
         <v>13</v>
@@ -6337,30 +6649,30 @@
         <v>13</v>
       </c>
       <c r="F101" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="G101" t="s">
         <v>15</v>
       </c>
       <c r="H101" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I101" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="J101" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="K101" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B102" t="s">
-        <v>13</v>
+        <v>332</v>
       </c>
       <c r="C102" t="s">
         <v>13</v>
@@ -6372,30 +6684,30 @@
         <v>13</v>
       </c>
       <c r="F102" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="G102" t="s">
         <v>15</v>
       </c>
       <c r="H102" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I102" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="J102" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="K102" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="B103" t="s">
-        <v>13</v>
+        <v>599</v>
       </c>
       <c r="C103" t="s">
         <v>13</v>
@@ -6407,30 +6719,30 @@
         <v>13</v>
       </c>
       <c r="F103" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="G103" t="s">
         <v>15</v>
       </c>
       <c r="H103" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="I103" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="J103" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="K103" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B104" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C104" t="s">
         <v>13</v>
@@ -6442,30 +6754,30 @@
         <v>13</v>
       </c>
       <c r="F104" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="G104" t="s">
         <v>15</v>
       </c>
       <c r="H104" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="I104" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="J104" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="K104" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="B105" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C105" t="s">
         <v>13</v>
@@ -6477,30 +6789,30 @@
         <v>13</v>
       </c>
       <c r="F105" t="s">
+        <v>612</v>
+      </c>
+      <c r="G105" t="s">
+        <v>15</v>
+      </c>
+      <c r="H105" t="s">
         <v>607</v>
       </c>
-      <c r="G105" t="s">
-        <v>15</v>
-      </c>
-      <c r="H105" t="s">
-        <v>577</v>
-      </c>
       <c r="I105" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="J105" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="K105" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="B106" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C106" t="s">
         <v>13</v>
@@ -6512,30 +6824,30 @@
         <v>13</v>
       </c>
       <c r="F106" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="G106" t="s">
         <v>15</v>
       </c>
       <c r="H106" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="I106" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="J106" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="K106" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="B107" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C107" t="s">
         <v>13</v>
@@ -6547,30 +6859,30 @@
         <v>13</v>
       </c>
       <c r="F107" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="G107" t="s">
         <v>15</v>
       </c>
       <c r="H107" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="I107" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="J107" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="K107" t="s">
-        <v>620</v>
+        <v>214</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B108" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C108" t="s">
         <v>13</v>
@@ -6582,30 +6894,30 @@
         <v>13</v>
       </c>
       <c r="F108" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="G108" t="s">
         <v>15</v>
       </c>
       <c r="H108" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="I108" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="J108" t="s">
-        <v>624</v>
+        <v>13</v>
       </c>
       <c r="K108" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B109" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C109" t="s">
         <v>13</v>
@@ -6617,30 +6929,30 @@
         <v>13</v>
       </c>
       <c r="F109" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="G109" t="s">
         <v>15</v>
       </c>
       <c r="H109" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="I109" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="J109" t="s">
-        <v>629</v>
+        <v>13</v>
       </c>
       <c r="K109" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B110" t="s">
-        <v>13</v>
+        <v>605</v>
       </c>
       <c r="C110" t="s">
         <v>13</v>
@@ -6652,30 +6964,30 @@
         <v>13</v>
       </c>
       <c r="F110" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="G110" t="s">
         <v>15</v>
       </c>
       <c r="H110" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="I110" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="J110" t="s">
-        <v>634</v>
+        <v>13</v>
       </c>
       <c r="K110" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B111" t="s">
-        <v>109</v>
+        <v>605</v>
       </c>
       <c r="C111" t="s">
         <v>13</v>
@@ -6687,13 +6999,13 @@
         <v>13</v>
       </c>
       <c r="F111" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="G111" t="s">
         <v>15</v>
       </c>
       <c r="H111" t="s">
-        <v>638</v>
+        <v>607</v>
       </c>
       <c r="I111" t="s">
         <v>639</v>
@@ -6710,252 +7022,252 @@
         <v>642</v>
       </c>
       <c r="B112" t="s">
+        <v>605</v>
+      </c>
+      <c r="C112" t="s">
+        <v>13</v>
+      </c>
+      <c r="D112" t="s">
+        <v>13</v>
+      </c>
+      <c r="E112" t="s">
+        <v>13</v>
+      </c>
+      <c r="F112" t="s">
         <v>643</v>
       </c>
-      <c r="C112" t="s">
-        <v>13</v>
-      </c>
-      <c r="D112" t="s">
-        <v>13</v>
-      </c>
-      <c r="E112" t="s">
-        <v>13</v>
-      </c>
-      <c r="F112" t="s">
+      <c r="G112" t="s">
+        <v>15</v>
+      </c>
+      <c r="H112" t="s">
+        <v>607</v>
+      </c>
+      <c r="I112" t="s">
         <v>644</v>
       </c>
-      <c r="G112" t="s">
-        <v>15</v>
-      </c>
-      <c r="H112" t="s">
-        <v>379</v>
-      </c>
-      <c r="I112" t="s">
+      <c r="J112" t="s">
         <v>645</v>
       </c>
-      <c r="J112" t="s">
+      <c r="K112" t="s">
         <v>646</v>
-      </c>
-      <c r="K112" t="s">
-        <v>647</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
+        <v>647</v>
+      </c>
+      <c r="B113" t="s">
+        <v>605</v>
+      </c>
+      <c r="C113" t="s">
+        <v>13</v>
+      </c>
+      <c r="D113" t="s">
+        <v>13</v>
+      </c>
+      <c r="E113" t="s">
+        <v>13</v>
+      </c>
+      <c r="F113" t="s">
         <v>648</v>
       </c>
-      <c r="B113" t="s">
-        <v>495</v>
-      </c>
-      <c r="C113" t="s">
-        <v>13</v>
-      </c>
-      <c r="D113" t="s">
-        <v>13</v>
-      </c>
-      <c r="E113" t="s">
-        <v>13</v>
-      </c>
-      <c r="F113" t="s">
+      <c r="G113" t="s">
+        <v>15</v>
+      </c>
+      <c r="H113" t="s">
+        <v>607</v>
+      </c>
+      <c r="I113" t="s">
         <v>649</v>
       </c>
-      <c r="G113" t="s">
-        <v>15</v>
-      </c>
-      <c r="H113" t="s">
-        <v>379</v>
-      </c>
-      <c r="I113" t="s">
+      <c r="J113" t="s">
+        <v>13</v>
+      </c>
+      <c r="K113" t="s">
         <v>650</v>
-      </c>
-      <c r="J113" t="s">
-        <v>651</v>
-      </c>
-      <c r="K113" t="s">
-        <v>652</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>651</v>
+      </c>
+      <c r="B114" t="s">
+        <v>605</v>
+      </c>
+      <c r="C114" t="s">
+        <v>13</v>
+      </c>
+      <c r="D114" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" t="s">
+        <v>13</v>
+      </c>
+      <c r="F114" t="s">
+        <v>652</v>
+      </c>
+      <c r="G114" t="s">
+        <v>15</v>
+      </c>
+      <c r="H114" t="s">
+        <v>607</v>
+      </c>
+      <c r="I114" t="s">
         <v>653</v>
       </c>
-      <c r="B114" t="s">
-        <v>495</v>
-      </c>
-      <c r="C114" t="s">
-        <v>13</v>
-      </c>
-      <c r="D114" t="s">
-        <v>13</v>
-      </c>
-      <c r="E114" t="s">
-        <v>13</v>
-      </c>
-      <c r="F114" t="s">
+      <c r="J114" t="s">
         <v>654</v>
       </c>
-      <c r="G114" t="s">
-        <v>15</v>
-      </c>
-      <c r="H114" t="s">
-        <v>379</v>
-      </c>
-      <c r="I114" t="s">
+      <c r="K114" t="s">
         <v>655</v>
-      </c>
-      <c r="J114" t="s">
-        <v>656</v>
-      </c>
-      <c r="K114" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>656</v>
+      </c>
+      <c r="B115" t="s">
+        <v>605</v>
+      </c>
+      <c r="C115" t="s">
+        <v>13</v>
+      </c>
+      <c r="D115" t="s">
+        <v>13</v>
+      </c>
+      <c r="E115" t="s">
+        <v>13</v>
+      </c>
+      <c r="F115" t="s">
+        <v>657</v>
+      </c>
+      <c r="G115" t="s">
+        <v>15</v>
+      </c>
+      <c r="H115" t="s">
+        <v>607</v>
+      </c>
+      <c r="I115" t="s">
         <v>658</v>
       </c>
-      <c r="B115" t="s">
-        <v>495</v>
-      </c>
-      <c r="C115" t="s">
-        <v>13</v>
-      </c>
-      <c r="D115" t="s">
-        <v>13</v>
-      </c>
-      <c r="E115" t="s">
-        <v>13</v>
-      </c>
-      <c r="F115" t="s">
+      <c r="J115" t="s">
         <v>659</v>
       </c>
-      <c r="G115" t="s">
-        <v>15</v>
-      </c>
-      <c r="H115" t="s">
-        <v>379</v>
-      </c>
-      <c r="I115" t="s">
+      <c r="K115" t="s">
         <v>660</v>
-      </c>
-      <c r="J115" t="s">
-        <v>661</v>
-      </c>
-      <c r="K115" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
+        <v>661</v>
+      </c>
+      <c r="B116" t="s">
+        <v>605</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116" t="s">
+        <v>13</v>
+      </c>
+      <c r="E116" t="s">
+        <v>13</v>
+      </c>
+      <c r="F116" t="s">
+        <v>662</v>
+      </c>
+      <c r="G116" t="s">
+        <v>15</v>
+      </c>
+      <c r="H116" t="s">
+        <v>607</v>
+      </c>
+      <c r="I116" t="s">
         <v>663</v>
       </c>
-      <c r="B116" t="s">
+      <c r="J116" t="s">
+        <v>13</v>
+      </c>
+      <c r="K116" t="s">
         <v>664</v>
-      </c>
-      <c r="C116" t="s">
-        <v>13</v>
-      </c>
-      <c r="D116" t="s">
-        <v>13</v>
-      </c>
-      <c r="E116" t="s">
-        <v>13</v>
-      </c>
-      <c r="F116" t="s">
-        <v>665</v>
-      </c>
-      <c r="G116" t="s">
-        <v>15</v>
-      </c>
-      <c r="H116" t="s">
-        <v>379</v>
-      </c>
-      <c r="I116" t="s">
-        <v>666</v>
-      </c>
-      <c r="J116" t="s">
-        <v>667</v>
-      </c>
-      <c r="K116" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
+        <v>665</v>
+      </c>
+      <c r="B117" t="s">
+        <v>605</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" t="s">
+        <v>13</v>
+      </c>
+      <c r="F117" t="s">
+        <v>666</v>
+      </c>
+      <c r="G117" t="s">
+        <v>15</v>
+      </c>
+      <c r="H117" t="s">
+        <v>607</v>
+      </c>
+      <c r="I117" t="s">
+        <v>667</v>
+      </c>
+      <c r="J117" t="s">
+        <v>668</v>
+      </c>
+      <c r="K117" t="s">
         <v>669</v>
-      </c>
-      <c r="B117" t="s">
-        <v>495</v>
-      </c>
-      <c r="C117" t="s">
-        <v>13</v>
-      </c>
-      <c r="D117" t="s">
-        <v>13</v>
-      </c>
-      <c r="E117" t="s">
-        <v>13</v>
-      </c>
-      <c r="F117" t="s">
-        <v>670</v>
-      </c>
-      <c r="G117" t="s">
-        <v>15</v>
-      </c>
-      <c r="H117" t="s">
-        <v>379</v>
-      </c>
-      <c r="I117" t="s">
-        <v>671</v>
-      </c>
-      <c r="J117" t="s">
-        <v>672</v>
-      </c>
-      <c r="K117" t="s">
-        <v>673</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
+        <v>670</v>
+      </c>
+      <c r="B118" t="s">
+        <v>605</v>
+      </c>
+      <c r="C118" t="s">
+        <v>13</v>
+      </c>
+      <c r="D118" t="s">
+        <v>13</v>
+      </c>
+      <c r="E118" t="s">
+        <v>13</v>
+      </c>
+      <c r="F118" t="s">
+        <v>671</v>
+      </c>
+      <c r="G118" t="s">
+        <v>15</v>
+      </c>
+      <c r="H118" t="s">
+        <v>607</v>
+      </c>
+      <c r="I118" t="s">
+        <v>672</v>
+      </c>
+      <c r="J118" t="s">
+        <v>673</v>
+      </c>
+      <c r="K118" t="s">
         <v>674</v>
-      </c>
-      <c r="B118" t="s">
-        <v>675</v>
-      </c>
-      <c r="C118" t="s">
-        <v>13</v>
-      </c>
-      <c r="D118" t="s">
-        <v>13</v>
-      </c>
-      <c r="E118" t="s">
-        <v>13</v>
-      </c>
-      <c r="F118" t="s">
-        <v>676</v>
-      </c>
-      <c r="G118" t="s">
-        <v>15</v>
-      </c>
-      <c r="H118" t="s">
-        <v>379</v>
-      </c>
-      <c r="I118" t="s">
-        <v>677</v>
-      </c>
-      <c r="J118" t="s">
-        <v>678</v>
-      </c>
-      <c r="K118" t="s">
-        <v>679</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>680</v>
+        <v>675</v>
       </c>
       <c r="B119" t="s">
-        <v>643</v>
+        <v>605</v>
       </c>
       <c r="C119" t="s">
         <v>13</v>
@@ -6967,30 +7279,30 @@
         <v>13</v>
       </c>
       <c r="F119" t="s">
-        <v>681</v>
+        <v>676</v>
       </c>
       <c r="G119" t="s">
         <v>15</v>
       </c>
       <c r="H119" t="s">
-        <v>379</v>
+        <v>607</v>
       </c>
       <c r="I119" t="s">
-        <v>682</v>
+        <v>677</v>
       </c>
       <c r="J119" t="s">
-        <v>683</v>
+        <v>13</v>
       </c>
       <c r="K119" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
       <c r="B120" t="s">
-        <v>479</v>
+        <v>13</v>
       </c>
       <c r="C120" t="s">
         <v>13</v>
@@ -7002,30 +7314,30 @@
         <v>13</v>
       </c>
       <c r="F120" t="s">
-        <v>686</v>
+        <v>680</v>
       </c>
       <c r="G120" t="s">
         <v>15</v>
       </c>
       <c r="H120" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I120" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="J120" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="K120" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B121" t="s">
-        <v>495</v>
+        <v>13</v>
       </c>
       <c r="C121" t="s">
         <v>13</v>
@@ -7037,30 +7349,30 @@
         <v>13</v>
       </c>
       <c r="F121" t="s">
-        <v>691</v>
+        <v>686</v>
       </c>
       <c r="G121" t="s">
         <v>15</v>
       </c>
       <c r="H121" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I121" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="J121" t="s">
-        <v>693</v>
+        <v>688</v>
       </c>
       <c r="K121" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="B122" t="s">
-        <v>696</v>
+        <v>13</v>
       </c>
       <c r="C122" t="s">
         <v>13</v>
@@ -7072,30 +7384,30 @@
         <v>13</v>
       </c>
       <c r="F122" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="G122" t="s">
         <v>15</v>
       </c>
       <c r="H122" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I122" t="s">
-        <v>698</v>
+        <v>692</v>
       </c>
       <c r="J122" t="s">
-        <v>699</v>
+        <v>693</v>
       </c>
       <c r="K122" t="s">
-        <v>700</v>
+        <v>694</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="B123" t="s">
-        <v>702</v>
+        <v>13</v>
       </c>
       <c r="C123" t="s">
         <v>13</v>
@@ -7107,30 +7419,30 @@
         <v>13</v>
       </c>
       <c r="F123" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
       <c r="G123" t="s">
         <v>15</v>
       </c>
       <c r="H123" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I123" t="s">
-        <v>704</v>
+        <v>697</v>
       </c>
       <c r="J123" t="s">
-        <v>705</v>
+        <v>698</v>
       </c>
       <c r="K123" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>707</v>
+        <v>700</v>
       </c>
       <c r="B124" t="s">
-        <v>495</v>
+        <v>13</v>
       </c>
       <c r="C124" t="s">
         <v>13</v>
@@ -7142,30 +7454,30 @@
         <v>13</v>
       </c>
       <c r="F124" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
       <c r="G124" t="s">
         <v>15</v>
       </c>
       <c r="H124" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I124" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="J124" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
       <c r="K124" t="s">
-        <v>711</v>
+        <v>704</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
       <c r="B125" t="s">
-        <v>643</v>
+        <v>13</v>
       </c>
       <c r="C125" t="s">
         <v>13</v>
@@ -7177,30 +7489,30 @@
         <v>13</v>
       </c>
       <c r="F125" t="s">
-        <v>713</v>
+        <v>706</v>
       </c>
       <c r="G125" t="s">
         <v>15</v>
       </c>
       <c r="H125" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I125" t="s">
-        <v>714</v>
+        <v>707</v>
       </c>
       <c r="J125" t="s">
-        <v>715</v>
+        <v>708</v>
       </c>
       <c r="K125" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>717</v>
+        <v>710</v>
       </c>
       <c r="B126" t="s">
-        <v>718</v>
+        <v>13</v>
       </c>
       <c r="C126" t="s">
         <v>13</v>
@@ -7212,30 +7524,30 @@
         <v>13</v>
       </c>
       <c r="F126" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="G126" t="s">
         <v>15</v>
       </c>
       <c r="H126" t="s">
-        <v>367</v>
+        <v>681</v>
       </c>
       <c r="I126" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
       <c r="J126" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
       <c r="K126" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="B127" t="s">
-        <v>724</v>
+        <v>13</v>
       </c>
       <c r="C127" t="s">
         <v>13</v>
@@ -7247,30 +7559,30 @@
         <v>13</v>
       </c>
       <c r="F127" t="s">
-        <v>725</v>
+        <v>716</v>
       </c>
       <c r="G127" t="s">
         <v>15</v>
       </c>
       <c r="H127" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I127" t="s">
-        <v>726</v>
+        <v>717</v>
       </c>
       <c r="J127" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="K127" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="B128" t="s">
-        <v>495</v>
+        <v>13</v>
       </c>
       <c r="C128" t="s">
         <v>13</v>
@@ -7282,30 +7594,30 @@
         <v>13</v>
       </c>
       <c r="F128" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
       <c r="G128" t="s">
         <v>15</v>
       </c>
       <c r="H128" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I128" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="J128" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
       <c r="K128" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B129" t="s">
-        <v>643</v>
+        <v>13</v>
       </c>
       <c r="C129" t="s">
         <v>13</v>
@@ -7317,30 +7629,30 @@
         <v>13</v>
       </c>
       <c r="F129" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
       <c r="G129" t="s">
         <v>15</v>
       </c>
       <c r="H129" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I129" t="s">
-        <v>735</v>
+        <v>727</v>
       </c>
       <c r="J129" t="s">
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="K129" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="B130" t="s">
-        <v>495</v>
+        <v>13</v>
       </c>
       <c r="C130" t="s">
         <v>13</v>
@@ -7352,30 +7664,30 @@
         <v>13</v>
       </c>
       <c r="F130" t="s">
-        <v>739</v>
+        <v>731</v>
       </c>
       <c r="G130" t="s">
         <v>15</v>
       </c>
       <c r="H130" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I130" t="s">
-        <v>740</v>
+        <v>732</v>
       </c>
       <c r="J130" t="s">
-        <v>741</v>
+        <v>733</v>
       </c>
       <c r="K130" t="s">
-        <v>742</v>
+        <v>734</v>
       </c>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>743</v>
+        <v>735</v>
       </c>
       <c r="B131" t="s">
-        <v>495</v>
+        <v>13</v>
       </c>
       <c r="C131" t="s">
         <v>13</v>
@@ -7387,30 +7699,30 @@
         <v>13</v>
       </c>
       <c r="F131" t="s">
-        <v>744</v>
+        <v>736</v>
       </c>
       <c r="G131" t="s">
         <v>15</v>
       </c>
       <c r="H131" t="s">
-        <v>379</v>
+        <v>681</v>
       </c>
       <c r="I131" t="s">
-        <v>745</v>
+        <v>737</v>
       </c>
       <c r="J131" t="s">
-        <v>746</v>
+        <v>738</v>
       </c>
       <c r="K131" t="s">
-        <v>747</v>
+        <v>739</v>
       </c>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="B132" t="s">
-        <v>643</v>
+        <v>109</v>
       </c>
       <c r="C132" t="s">
         <v>13</v>
@@ -7422,30 +7734,30 @@
         <v>13</v>
       </c>
       <c r="F132" t="s">
-        <v>749</v>
+        <v>741</v>
       </c>
       <c r="G132" t="s">
         <v>15</v>
       </c>
       <c r="H132" t="s">
-        <v>379</v>
+        <v>742</v>
       </c>
       <c r="I132" t="s">
-        <v>750</v>
+        <v>743</v>
       </c>
       <c r="J132" t="s">
-        <v>751</v>
+        <v>744</v>
       </c>
       <c r="K132" t="s">
-        <v>752</v>
+        <v>745</v>
       </c>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>753</v>
+        <v>746</v>
       </c>
       <c r="B133" t="s">
-        <v>109</v>
+        <v>747</v>
       </c>
       <c r="C133" t="s">
         <v>13</v>
@@ -7457,30 +7769,30 @@
         <v>13</v>
       </c>
       <c r="F133" t="s">
-        <v>754</v>
+        <v>748</v>
       </c>
       <c r="G133" t="s">
         <v>15</v>
       </c>
       <c r="H133" t="s">
-        <v>424</v>
+        <v>484</v>
       </c>
       <c r="I133" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="J133" t="s">
-        <v>756</v>
+        <v>750</v>
       </c>
       <c r="K133" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>758</v>
+        <v>752</v>
       </c>
       <c r="B134" t="s">
-        <v>109</v>
+        <v>599</v>
       </c>
       <c r="C134" t="s">
         <v>13</v>
@@ -7492,30 +7804,30 @@
         <v>13</v>
       </c>
       <c r="F134" t="s">
-        <v>759</v>
+        <v>753</v>
       </c>
       <c r="G134" t="s">
         <v>15</v>
       </c>
       <c r="H134" t="s">
-        <v>424</v>
+        <v>484</v>
       </c>
       <c r="I134" t="s">
-        <v>760</v>
+        <v>754</v>
       </c>
       <c r="J134" t="s">
-        <v>761</v>
+        <v>755</v>
       </c>
       <c r="K134" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="B135" t="s">
-        <v>109</v>
+        <v>599</v>
       </c>
       <c r="C135" t="s">
         <v>13</v>
@@ -7527,30 +7839,30 @@
         <v>13</v>
       </c>
       <c r="F135" t="s">
-        <v>764</v>
+        <v>758</v>
       </c>
       <c r="G135" t="s">
         <v>15</v>
       </c>
       <c r="H135" t="s">
-        <v>424</v>
+        <v>484</v>
       </c>
       <c r="I135" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="J135" t="s">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="K135" t="s">
-        <v>767</v>
+        <v>761</v>
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>768</v>
+        <v>762</v>
       </c>
       <c r="B136" t="s">
-        <v>109</v>
+        <v>599</v>
       </c>
       <c r="C136" t="s">
         <v>13</v>
@@ -7562,30 +7874,30 @@
         <v>13</v>
       </c>
       <c r="F136" t="s">
-        <v>769</v>
+        <v>763</v>
       </c>
       <c r="G136" t="s">
         <v>15</v>
       </c>
       <c r="H136" t="s">
-        <v>424</v>
+        <v>484</v>
       </c>
       <c r="I136" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="J136" t="s">
-        <v>771</v>
+        <v>765</v>
       </c>
       <c r="K136" t="s">
-        <v>772</v>
+        <v>766</v>
       </c>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>773</v>
+        <v>767</v>
       </c>
       <c r="B137" t="s">
-        <v>109</v>
+        <v>768</v>
       </c>
       <c r="C137" t="s">
         <v>13</v>
@@ -7597,30 +7909,30 @@
         <v>13</v>
       </c>
       <c r="F137" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="G137" t="s">
         <v>15</v>
       </c>
       <c r="H137" t="s">
-        <v>638</v>
+        <v>484</v>
       </c>
       <c r="I137" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="J137" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
       <c r="K137" t="s">
-        <v>777</v>
+        <v>772</v>
       </c>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="B138" t="s">
-        <v>109</v>
+        <v>599</v>
       </c>
       <c r="C138" t="s">
         <v>13</v>
@@ -7632,127 +7944,862 @@
         <v>13</v>
       </c>
       <c r="F138" t="s">
-        <v>779</v>
+        <v>774</v>
       </c>
       <c r="G138" t="s">
         <v>15</v>
       </c>
       <c r="H138" t="s">
-        <v>424</v>
+        <v>484</v>
       </c>
       <c r="I138" t="s">
-        <v>780</v>
+        <v>775</v>
       </c>
       <c r="J138" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="K138" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
+        <v>778</v>
+      </c>
+      <c r="B139" t="s">
+        <v>779</v>
+      </c>
+      <c r="C139" t="s">
+        <v>13</v>
+      </c>
+      <c r="D139" t="s">
+        <v>13</v>
+      </c>
+      <c r="E139" t="s">
+        <v>13</v>
+      </c>
+      <c r="F139" t="s">
+        <v>780</v>
+      </c>
+      <c r="G139" t="s">
+        <v>15</v>
+      </c>
+      <c r="H139" t="s">
+        <v>484</v>
+      </c>
+      <c r="I139" t="s">
+        <v>781</v>
+      </c>
+      <c r="J139" t="s">
+        <v>782</v>
+      </c>
+      <c r="K139" t="s">
         <v>783</v>
-      </c>
-      <c r="B139" t="s">
-        <v>784</v>
-      </c>
-      <c r="C139" t="s">
-        <v>451</v>
-      </c>
-      <c r="D139" t="s">
-        <v>13</v>
-      </c>
-      <c r="E139" t="s">
-        <v>785</v>
-      </c>
-      <c r="F139" t="s">
-        <v>786</v>
-      </c>
-      <c r="G139" t="s">
-        <v>15</v>
-      </c>
-      <c r="H139" t="s">
-        <v>467</v>
-      </c>
-      <c r="I139" t="s">
-        <v>787</v>
-      </c>
-      <c r="J139" t="s">
-        <v>788</v>
-      </c>
-      <c r="K139" t="s">
-        <v>789</v>
       </c>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>790</v>
+        <v>784</v>
       </c>
       <c r="B140" t="s">
-        <v>784</v>
+        <v>747</v>
       </c>
       <c r="C140" t="s">
-        <v>458</v>
+        <v>13</v>
       </c>
       <c r="D140" t="s">
         <v>13</v>
       </c>
       <c r="E140" t="s">
+        <v>13</v>
+      </c>
+      <c r="F140" t="s">
         <v>785</v>
       </c>
-      <c r="F140" t="s">
-        <v>791</v>
-      </c>
       <c r="G140" t="s">
         <v>15</v>
       </c>
       <c r="H140" t="s">
-        <v>467</v>
+        <v>484</v>
       </c>
       <c r="I140" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="J140" t="s">
-        <v>793</v>
+        <v>787</v>
       </c>
       <c r="K140" t="s">
-        <v>794</v>
+        <v>788</v>
       </c>
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
+        <v>789</v>
+      </c>
+      <c r="B141" t="s">
+        <v>332</v>
+      </c>
+      <c r="C141" t="s">
+        <v>13</v>
+      </c>
+      <c r="D141" t="s">
+        <v>13</v>
+      </c>
+      <c r="E141" t="s">
+        <v>13</v>
+      </c>
+      <c r="F141" t="s">
+        <v>790</v>
+      </c>
+      <c r="G141" t="s">
+        <v>15</v>
+      </c>
+      <c r="H141" t="s">
+        <v>484</v>
+      </c>
+      <c r="I141" t="s">
+        <v>791</v>
+      </c>
+      <c r="J141" t="s">
+        <v>792</v>
+      </c>
+      <c r="K141" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>794</v>
+      </c>
+      <c r="B142" t="s">
+        <v>599</v>
+      </c>
+      <c r="C142" t="s">
+        <v>13</v>
+      </c>
+      <c r="D142" t="s">
+        <v>13</v>
+      </c>
+      <c r="E142" t="s">
+        <v>13</v>
+      </c>
+      <c r="F142" t="s">
         <v>795</v>
       </c>
-      <c r="B141" t="s">
+      <c r="G142" t="s">
+        <v>15</v>
+      </c>
+      <c r="H142" t="s">
+        <v>484</v>
+      </c>
+      <c r="I142" t="s">
         <v>796</v>
       </c>
-      <c r="C141" t="s">
+      <c r="J142" t="s">
         <v>797</v>
       </c>
-      <c r="D141" t="s">
-        <v>13</v>
-      </c>
-      <c r="E141" t="s">
+      <c r="K142" t="s">
         <v>798</v>
       </c>
-      <c r="F141" t="s">
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>799</v>
       </c>
-      <c r="G141" t="s">
-        <v>15</v>
-      </c>
-      <c r="H141" t="s">
-        <v>467</v>
-      </c>
-      <c r="I141" t="s">
+      <c r="B143" t="s">
         <v>800</v>
       </c>
-      <c r="J141" t="s">
+      <c r="C143" t="s">
+        <v>13</v>
+      </c>
+      <c r="D143" t="s">
+        <v>13</v>
+      </c>
+      <c r="E143" t="s">
+        <v>13</v>
+      </c>
+      <c r="F143" t="s">
         <v>801</v>
       </c>
-      <c r="K141" t="s">
+      <c r="G143" t="s">
+        <v>15</v>
+      </c>
+      <c r="H143" t="s">
+        <v>484</v>
+      </c>
+      <c r="I143" t="s">
         <v>802</v>
+      </c>
+      <c r="J143" t="s">
+        <v>803</v>
+      </c>
+      <c r="K143" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>805</v>
+      </c>
+      <c r="B144" t="s">
+        <v>806</v>
+      </c>
+      <c r="C144" t="s">
+        <v>13</v>
+      </c>
+      <c r="D144" t="s">
+        <v>13</v>
+      </c>
+      <c r="E144" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144" t="s">
+        <v>807</v>
+      </c>
+      <c r="G144" t="s">
+        <v>15</v>
+      </c>
+      <c r="H144" t="s">
+        <v>484</v>
+      </c>
+      <c r="I144" t="s">
+        <v>808</v>
+      </c>
+      <c r="J144" t="s">
+        <v>809</v>
+      </c>
+      <c r="K144" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>811</v>
+      </c>
+      <c r="B145" t="s">
+        <v>599</v>
+      </c>
+      <c r="C145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D145" t="s">
+        <v>13</v>
+      </c>
+      <c r="E145" t="s">
+        <v>13</v>
+      </c>
+      <c r="F145" t="s">
+        <v>812</v>
+      </c>
+      <c r="G145" t="s">
+        <v>15</v>
+      </c>
+      <c r="H145" t="s">
+        <v>484</v>
+      </c>
+      <c r="I145" t="s">
+        <v>813</v>
+      </c>
+      <c r="J145" t="s">
+        <v>814</v>
+      </c>
+      <c r="K145" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>816</v>
+      </c>
+      <c r="B146" t="s">
+        <v>747</v>
+      </c>
+      <c r="C146" t="s">
+        <v>13</v>
+      </c>
+      <c r="D146" t="s">
+        <v>13</v>
+      </c>
+      <c r="E146" t="s">
+        <v>13</v>
+      </c>
+      <c r="F146" t="s">
+        <v>817</v>
+      </c>
+      <c r="G146" t="s">
+        <v>15</v>
+      </c>
+      <c r="H146" t="s">
+        <v>484</v>
+      </c>
+      <c r="I146" t="s">
+        <v>818</v>
+      </c>
+      <c r="J146" t="s">
+        <v>819</v>
+      </c>
+      <c r="K146" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>821</v>
+      </c>
+      <c r="B147" t="s">
+        <v>822</v>
+      </c>
+      <c r="C147" t="s">
+        <v>13</v>
+      </c>
+      <c r="D147" t="s">
+        <v>13</v>
+      </c>
+      <c r="E147" t="s">
+        <v>13</v>
+      </c>
+      <c r="F147" t="s">
+        <v>823</v>
+      </c>
+      <c r="G147" t="s">
+        <v>15</v>
+      </c>
+      <c r="H147" t="s">
+        <v>472</v>
+      </c>
+      <c r="I147" t="s">
+        <v>824</v>
+      </c>
+      <c r="J147" t="s">
+        <v>825</v>
+      </c>
+      <c r="K147" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>827</v>
+      </c>
+      <c r="B148" t="s">
+        <v>828</v>
+      </c>
+      <c r="C148" t="s">
+        <v>13</v>
+      </c>
+      <c r="D148" t="s">
+        <v>13</v>
+      </c>
+      <c r="E148" t="s">
+        <v>13</v>
+      </c>
+      <c r="F148" t="s">
+        <v>829</v>
+      </c>
+      <c r="G148" t="s">
+        <v>15</v>
+      </c>
+      <c r="H148" t="s">
+        <v>484</v>
+      </c>
+      <c r="I148" t="s">
+        <v>830</v>
+      </c>
+      <c r="J148" t="s">
+        <v>825</v>
+      </c>
+      <c r="K148" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>832</v>
+      </c>
+      <c r="B149" t="s">
+        <v>599</v>
+      </c>
+      <c r="C149" t="s">
+        <v>13</v>
+      </c>
+      <c r="D149" t="s">
+        <v>13</v>
+      </c>
+      <c r="E149" t="s">
+        <v>13</v>
+      </c>
+      <c r="F149" t="s">
+        <v>833</v>
+      </c>
+      <c r="G149" t="s">
+        <v>15</v>
+      </c>
+      <c r="H149" t="s">
+        <v>484</v>
+      </c>
+      <c r="I149" t="s">
+        <v>834</v>
+      </c>
+      <c r="J149" t="s">
+        <v>835</v>
+      </c>
+      <c r="K149" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>837</v>
+      </c>
+      <c r="B150" t="s">
+        <v>747</v>
+      </c>
+      <c r="C150" t="s">
+        <v>13</v>
+      </c>
+      <c r="D150" t="s">
+        <v>13</v>
+      </c>
+      <c r="E150" t="s">
+        <v>13</v>
+      </c>
+      <c r="F150" t="s">
+        <v>838</v>
+      </c>
+      <c r="G150" t="s">
+        <v>15</v>
+      </c>
+      <c r="H150" t="s">
+        <v>484</v>
+      </c>
+      <c r="I150" t="s">
+        <v>839</v>
+      </c>
+      <c r="J150" t="s">
+        <v>840</v>
+      </c>
+      <c r="K150" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>842</v>
+      </c>
+      <c r="B151" t="s">
+        <v>599</v>
+      </c>
+      <c r="C151" t="s">
+        <v>13</v>
+      </c>
+      <c r="D151" t="s">
+        <v>13</v>
+      </c>
+      <c r="E151" t="s">
+        <v>13</v>
+      </c>
+      <c r="F151" t="s">
+        <v>843</v>
+      </c>
+      <c r="G151" t="s">
+        <v>15</v>
+      </c>
+      <c r="H151" t="s">
+        <v>484</v>
+      </c>
+      <c r="I151" t="s">
+        <v>844</v>
+      </c>
+      <c r="J151" t="s">
+        <v>845</v>
+      </c>
+      <c r="K151" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>847</v>
+      </c>
+      <c r="B152" t="s">
+        <v>599</v>
+      </c>
+      <c r="C152" t="s">
+        <v>13</v>
+      </c>
+      <c r="D152" t="s">
+        <v>13</v>
+      </c>
+      <c r="E152" t="s">
+        <v>13</v>
+      </c>
+      <c r="F152" t="s">
+        <v>848</v>
+      </c>
+      <c r="G152" t="s">
+        <v>15</v>
+      </c>
+      <c r="H152" t="s">
+        <v>484</v>
+      </c>
+      <c r="I152" t="s">
+        <v>849</v>
+      </c>
+      <c r="J152" t="s">
+        <v>850</v>
+      </c>
+      <c r="K152" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>852</v>
+      </c>
+      <c r="B153" t="s">
+        <v>747</v>
+      </c>
+      <c r="C153" t="s">
+        <v>13</v>
+      </c>
+      <c r="D153" t="s">
+        <v>13</v>
+      </c>
+      <c r="E153" t="s">
+        <v>13</v>
+      </c>
+      <c r="F153" t="s">
+        <v>853</v>
+      </c>
+      <c r="G153" t="s">
+        <v>15</v>
+      </c>
+      <c r="H153" t="s">
+        <v>484</v>
+      </c>
+      <c r="I153" t="s">
+        <v>854</v>
+      </c>
+      <c r="J153" t="s">
+        <v>855</v>
+      </c>
+      <c r="K153" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>857</v>
+      </c>
+      <c r="B154" t="s">
+        <v>109</v>
+      </c>
+      <c r="C154" t="s">
+        <v>13</v>
+      </c>
+      <c r="D154" t="s">
+        <v>13</v>
+      </c>
+      <c r="E154" t="s">
+        <v>13</v>
+      </c>
+      <c r="F154" t="s">
+        <v>858</v>
+      </c>
+      <c r="G154" t="s">
+        <v>15</v>
+      </c>
+      <c r="H154" t="s">
+        <v>529</v>
+      </c>
+      <c r="I154" t="s">
+        <v>859</v>
+      </c>
+      <c r="J154" t="s">
+        <v>860</v>
+      </c>
+      <c r="K154" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>862</v>
+      </c>
+      <c r="B155" t="s">
+        <v>109</v>
+      </c>
+      <c r="C155" t="s">
+        <v>13</v>
+      </c>
+      <c r="D155" t="s">
+        <v>13</v>
+      </c>
+      <c r="E155" t="s">
+        <v>13</v>
+      </c>
+      <c r="F155" t="s">
+        <v>863</v>
+      </c>
+      <c r="G155" t="s">
+        <v>15</v>
+      </c>
+      <c r="H155" t="s">
+        <v>529</v>
+      </c>
+      <c r="I155" t="s">
+        <v>864</v>
+      </c>
+      <c r="J155" t="s">
+        <v>865</v>
+      </c>
+      <c r="K155" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>867</v>
+      </c>
+      <c r="B156" t="s">
+        <v>109</v>
+      </c>
+      <c r="C156" t="s">
+        <v>13</v>
+      </c>
+      <c r="D156" t="s">
+        <v>13</v>
+      </c>
+      <c r="E156" t="s">
+        <v>13</v>
+      </c>
+      <c r="F156" t="s">
+        <v>868</v>
+      </c>
+      <c r="G156" t="s">
+        <v>15</v>
+      </c>
+      <c r="H156" t="s">
+        <v>529</v>
+      </c>
+      <c r="I156" t="s">
+        <v>869</v>
+      </c>
+      <c r="J156" t="s">
+        <v>870</v>
+      </c>
+      <c r="K156" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>872</v>
+      </c>
+      <c r="B157" t="s">
+        <v>109</v>
+      </c>
+      <c r="C157" t="s">
+        <v>13</v>
+      </c>
+      <c r="D157" t="s">
+        <v>13</v>
+      </c>
+      <c r="E157" t="s">
+        <v>13</v>
+      </c>
+      <c r="F157" t="s">
+        <v>873</v>
+      </c>
+      <c r="G157" t="s">
+        <v>15</v>
+      </c>
+      <c r="H157" t="s">
+        <v>529</v>
+      </c>
+      <c r="I157" t="s">
+        <v>874</v>
+      </c>
+      <c r="J157" t="s">
+        <v>875</v>
+      </c>
+      <c r="K157" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>877</v>
+      </c>
+      <c r="B158" t="s">
+        <v>109</v>
+      </c>
+      <c r="C158" t="s">
+        <v>13</v>
+      </c>
+      <c r="D158" t="s">
+        <v>13</v>
+      </c>
+      <c r="E158" t="s">
+        <v>13</v>
+      </c>
+      <c r="F158" t="s">
+        <v>878</v>
+      </c>
+      <c r="G158" t="s">
+        <v>15</v>
+      </c>
+      <c r="H158" t="s">
+        <v>742</v>
+      </c>
+      <c r="I158" t="s">
+        <v>879</v>
+      </c>
+      <c r="J158" t="s">
+        <v>880</v>
+      </c>
+      <c r="K158" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>882</v>
+      </c>
+      <c r="B159" t="s">
+        <v>109</v>
+      </c>
+      <c r="C159" t="s">
+        <v>13</v>
+      </c>
+      <c r="D159" t="s">
+        <v>13</v>
+      </c>
+      <c r="E159" t="s">
+        <v>13</v>
+      </c>
+      <c r="F159" t="s">
+        <v>883</v>
+      </c>
+      <c r="G159" t="s">
+        <v>15</v>
+      </c>
+      <c r="H159" t="s">
+        <v>529</v>
+      </c>
+      <c r="I159" t="s">
+        <v>884</v>
+      </c>
+      <c r="J159" t="s">
+        <v>885</v>
+      </c>
+      <c r="K159" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>887</v>
+      </c>
+      <c r="B160" t="s">
+        <v>888</v>
+      </c>
+      <c r="C160" t="s">
+        <v>556</v>
+      </c>
+      <c r="D160" t="s">
+        <v>13</v>
+      </c>
+      <c r="E160" t="s">
+        <v>889</v>
+      </c>
+      <c r="F160" t="s">
+        <v>890</v>
+      </c>
+      <c r="G160" t="s">
+        <v>15</v>
+      </c>
+      <c r="H160" t="s">
+        <v>572</v>
+      </c>
+      <c r="I160" t="s">
+        <v>891</v>
+      </c>
+      <c r="J160" t="s">
+        <v>892</v>
+      </c>
+      <c r="K160" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>894</v>
+      </c>
+      <c r="B161" t="s">
+        <v>888</v>
+      </c>
+      <c r="C161" t="s">
+        <v>563</v>
+      </c>
+      <c r="D161" t="s">
+        <v>13</v>
+      </c>
+      <c r="E161" t="s">
+        <v>889</v>
+      </c>
+      <c r="F161" t="s">
+        <v>895</v>
+      </c>
+      <c r="G161" t="s">
+        <v>15</v>
+      </c>
+      <c r="H161" t="s">
+        <v>572</v>
+      </c>
+      <c r="I161" t="s">
+        <v>896</v>
+      </c>
+      <c r="J161" t="s">
+        <v>897</v>
+      </c>
+      <c r="K161" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>899</v>
+      </c>
+      <c r="B162" t="s">
+        <v>900</v>
+      </c>
+      <c r="C162" t="s">
+        <v>901</v>
+      </c>
+      <c r="D162" t="s">
+        <v>13</v>
+      </c>
+      <c r="E162" t="s">
+        <v>902</v>
+      </c>
+      <c r="F162" t="s">
+        <v>903</v>
+      </c>
+      <c r="G162" t="s">
+        <v>15</v>
+      </c>
+      <c r="H162" t="s">
+        <v>572</v>
+      </c>
+      <c r="I162" t="s">
+        <v>904</v>
+      </c>
+      <c r="J162" t="s">
+        <v>905</v>
+      </c>
+      <c r="K162" t="s">
+        <v>906</v>
       </c>
     </row>
   </sheetData>

</xml_diff>